<commit_message>
fix(trader): exit only on SL or target, correct portfolio history
Remove SIGNAL GONE and GAP DOWN exits so positions stay open until
stop-loss or target is hit. Reopen prematurely closed trades in the
portfolio and regenerate trade_log.xlsx. Add FII/DII date validation
in the scanner to avoid stale macro data before 16:30 IST.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/trade_log.xlsx
+++ b/trade_log.xlsx
@@ -48,18 +48,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -67,13 +67,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -443,68 +452,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Entry Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Exit Date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Entry ₹</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Exit ₹</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Exit Reason</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Macro</t>
         </is>
@@ -513,40 +528,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1417</v>
+        <v>1577.8</v>
       </c>
       <c r="E2" t="n">
-        <v>1415.7</v>
+        <v>1578.7</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>-91</v>
+        <v>63</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>56.7</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.09</v>
+        <v>0.06</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SIGNAL GONE</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
@@ -555,40 +575,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2109</v>
+        <v>14098</v>
       </c>
       <c r="E3" t="n">
-        <v>2103.8</v>
+        <v>14115</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>-244.4</v>
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>119</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.25</v>
+        <v>0.12</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SIGNAL GONE</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
@@ -597,40 +622,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABCAPITAL</t>
+          <t>FEDERALBNK</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>392</v>
+        <v>330.1</v>
       </c>
       <c r="E4" t="n">
-        <v>391.95</v>
+        <v>330.05</v>
       </c>
       <c r="F4" t="n">
-        <v>255</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>-12.75</v>
+        <v>302</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>-15.1</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SIGNAL GONE</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
@@ -639,40 +669,844 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IDFCFIRSTB</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>80</v>
+        <v>714.15</v>
       </c>
       <c r="E5" t="n">
-        <v>80.69</v>
+        <v>713.95</v>
       </c>
       <c r="F5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>862.5</v>
+        <v>140</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>-28</v>
       </c>
       <c r="H5" t="n">
-        <v>0.86</v>
+        <v>-0.03</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>SIGNAL GONE</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PAGEIND</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>40885</v>
+      </c>
+      <c r="E6" t="n">
+        <v>41370</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GODREJPROP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1852.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1866.6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>53</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>752.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1799.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1789.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>55</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>-539</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1385.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1350.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>-2512.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-2.52</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1455.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1465.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>68</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>680</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>959.85</v>
+      </c>
+      <c r="E11" t="n">
+        <v>952.15</v>
+      </c>
+      <c r="F11" t="n">
+        <v>104</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>-800.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AUBANK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1067.2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1051.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>93</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>-1469.4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>10468.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10805</v>
+      </c>
+      <c r="F13" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>3028.5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>TARGET HIT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>5207.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5440</v>
+      </c>
+      <c r="F14" t="n">
+        <v>19</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>4423.2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>TARGET HIT</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ABCAPITAL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>394.8</v>
+      </c>
+      <c r="E15" t="n">
+        <v>390.4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>252</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>-1108.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>26070</v>
+      </c>
+      <c r="E16" t="n">
+        <v>25785</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>-855</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-1.09</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3247</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3211.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>-1077</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5450</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5381.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>18</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>-1225.8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>151.72</v>
+      </c>
+      <c r="E19" t="n">
+        <v>150.19</v>
+      </c>
+      <c r="F19" t="n">
+        <v>659</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>-1008.27</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1120</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1155.25</v>
+      </c>
+      <c r="F20" t="n">
+        <v>89</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>3137.25</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>TARGET HIT</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>620.1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>610.45</v>
+      </c>
+      <c r="F21" t="n">
+        <v>161</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>-1553.65</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SL HIT</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NYKAA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>302</v>
+      </c>
+      <c r="E22" t="n">
+        <v>308.35</v>
+      </c>
+      <c r="F22" t="n">
+        <v>331</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>2101.85</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>TARGET HIT</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
@@ -689,14 +1523,488 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Entry Date</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Entry ₹</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>CMP ₹</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Invested ₹</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Unrealised ₹</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>SL ₹</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Target ₹</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1577.8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1578.7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+      <c r="F2" t="n">
+        <v>99401.39999999999</v>
+      </c>
+      <c r="G2" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1562.02</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1609.36</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>14098</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14115</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>98686</v>
+      </c>
+      <c r="G3" t="n">
+        <v>119</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I3" t="n">
+        <v>13957.02</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14379.96</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FEDERALBNK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>330.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>330.05</v>
+      </c>
+      <c r="E4" t="n">
+        <v>302</v>
+      </c>
+      <c r="F4" t="n">
+        <v>99690.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-15.1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="I4" t="n">
+        <v>326.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>714.15</v>
+      </c>
+      <c r="D5" t="n">
+        <v>713.95</v>
+      </c>
+      <c r="E5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F5" t="n">
+        <v>99981</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-28</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="I5" t="n">
+        <v>707.01</v>
+      </c>
+      <c r="J5" t="n">
+        <v>728.4299999999999</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PAGEIND</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>40885</v>
+      </c>
+      <c r="D6" t="n">
+        <v>41370</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>81770</v>
+      </c>
+      <c r="G6" t="n">
+        <v>970</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I6" t="n">
+        <v>40476.15</v>
+      </c>
+      <c r="J6" t="n">
+        <v>41702.7</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GODREJPROP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1852.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1866.6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F7" t="n">
+        <v>98177.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>752.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1833.88</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1889.45</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1799.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1789.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>55</v>
+      </c>
+      <c r="F8" t="n">
+        <v>98978</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-539</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1781.6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1835.59</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1385.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1350.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F9" t="n">
+        <v>99741.60000000001</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-2512.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-2.52</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1371.45</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1413.01</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1455.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1465.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>68</v>
+      </c>
+      <c r="F10" t="n">
+        <v>98967.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>680</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1440.85</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1484.51</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>959.85</v>
+      </c>
+      <c r="D11" t="n">
+        <v>952.15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>104</v>
+      </c>
+      <c r="F11" t="n">
+        <v>99824.39999999999</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-800.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="I11" t="n">
+        <v>950.25</v>
+      </c>
+      <c r="J11" t="n">
+        <v>979.05</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -709,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -722,37 +2030,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Win Rate %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Cumul P&amp;L ₹</t>
         </is>
@@ -761,26 +2069,76 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2941.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>514.35</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2941.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>903.1799999999999</v>
+      </c>
+      <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G2" t="n">
-        <v>514.35</v>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3844.68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>548.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4392.88</v>
       </c>
     </row>
   </sheetData>
@@ -794,12 +2152,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -807,37 +2165,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Win Rate %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Cumul P&amp;L ₹</t>
         </is>
@@ -850,22 +2208,47 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2941.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>514.35</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2941.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>W27 2026</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1451.38</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G2" t="n">
-        <v>514.35</v>
+      <c r="F3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4392.88</v>
       </c>
     </row>
   </sheetData>
@@ -884,7 +2267,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -892,37 +2275,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Win Rate %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Cumul P&amp;L ₹</t>
         </is>
@@ -935,22 +2318,22 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4392.88</v>
+      </c>
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>514.35</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>25</v>
+        <v>36.4</v>
       </c>
       <c r="G2" t="n">
-        <v>514.35</v>
+        <v>4392.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(portfolio): close positions that hit SL/target in price history
Re-audit reopened trades using hourly bars after the 15:15 IST entry
time. Close PAGEIND at target and four others at stop-loss; keep only
positions that never breached SL or target after entry.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/trade_log.xlsx
+++ b/trade_log.xlsx
@@ -716,12 +716,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PAGEIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -730,19 +730,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40885</v>
+        <v>1455.4</v>
       </c>
       <c r="E6" t="n">
-        <v>41370</v>
+        <v>1465.4</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>970</v>
+        <v>680</v>
       </c>
       <c r="H6" t="n">
-        <v>1.19</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -763,183 +763,183 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>AUBANK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="D7" t="n">
-        <v>1852.4</v>
+        <v>1067.2</v>
       </c>
       <c r="E7" t="n">
-        <v>1866.6</v>
+        <v>1051.4</v>
       </c>
       <c r="F7" t="n">
-        <v>53</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>752.6</v>
+        <v>93</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>-1469.4</v>
       </c>
       <c r="H7" t="n">
-        <v>0.77</v>
+        <v>-1.48</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="D8" t="n">
-        <v>1799.6</v>
+        <v>10468.5</v>
       </c>
       <c r="E8" t="n">
-        <v>1789.8</v>
+        <v>10805</v>
       </c>
       <c r="F8" t="n">
-        <v>55</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>-539</v>
+        <v>9</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>3028.5</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.54</v>
+        <v>3.21</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TARGET HIT</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="D9" t="n">
-        <v>1385.3</v>
+        <v>5207.2</v>
       </c>
       <c r="E9" t="n">
-        <v>1350.4</v>
+        <v>5440</v>
       </c>
       <c r="F9" t="n">
-        <v>72</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>-2512.8</v>
+        <v>19</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>4423.2</v>
       </c>
       <c r="H9" t="n">
-        <v>-2.52</v>
+        <v>4.47</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TARGET HIT</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ABCAPITAL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1455.4</v>
+        <v>394.8</v>
       </c>
       <c r="E10" t="n">
-        <v>1465.4</v>
+        <v>390.4</v>
       </c>
       <c r="F10" t="n">
-        <v>68</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>680</v>
+        <v>252</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>-1108.8</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6899999999999999</v>
+        <v>-1.11</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -951,42 +951,42 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>959.85</v>
+        <v>26070</v>
       </c>
       <c r="E11" t="n">
-        <v>952.15</v>
+        <v>25785</v>
       </c>
       <c r="F11" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-800.8</v>
+        <v>-855</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.8</v>
+        <v>-1.09</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -998,7 +998,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AUBANK</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1012,19 +1012,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1067.2</v>
+        <v>3247</v>
       </c>
       <c r="E12" t="n">
-        <v>1051.4</v>
+        <v>3211.1</v>
       </c>
       <c r="F12" t="n">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-1469.4</v>
+        <v>-1077</v>
       </c>
       <c r="H12" t="n">
-        <v>-1.48</v>
+        <v>-1.11</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1045,33 +1045,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>10468.5</v>
+        <v>5450</v>
       </c>
       <c r="E13" t="n">
-        <v>10805</v>
+        <v>5381.9</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>3028.5</v>
+        <v>18</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>-1225.8</v>
       </c>
       <c r="H13" t="n">
-        <v>3.21</v>
+        <v>-1.25</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>TARGET HIT</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1092,33 +1092,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5207.2</v>
+        <v>151.72</v>
       </c>
       <c r="E14" t="n">
-        <v>5440</v>
+        <v>150.19</v>
       </c>
       <c r="F14" t="n">
-        <v>19</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>4423.2</v>
+        <v>659</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>-1008.27</v>
       </c>
       <c r="H14" t="n">
-        <v>4.47</v>
+        <v>-1.01</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>TARGET HIT</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1139,33 +1139,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABCAPITAL</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>394.8</v>
+        <v>1120</v>
       </c>
       <c r="E15" t="n">
-        <v>390.4</v>
+        <v>1155.25</v>
       </c>
       <c r="F15" t="n">
-        <v>252</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>-1108.8</v>
+        <v>89</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>3137.25</v>
       </c>
       <c r="H15" t="n">
-        <v>-1.11</v>
+        <v>3.15</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>SL HIT</t>
+          <t>TARGET HIT</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1186,33 +1186,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>26070</v>
+        <v>620.1</v>
       </c>
       <c r="E16" t="n">
-        <v>25785</v>
+        <v>610.45</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>161</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>-855</v>
+        <v>-1553.65</v>
       </c>
       <c r="H16" t="n">
-        <v>-1.09</v>
+        <v>-1.56</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1233,33 +1233,33 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3247</v>
+        <v>302</v>
       </c>
       <c r="E17" t="n">
-        <v>3211.1</v>
+        <v>308.35</v>
       </c>
       <c r="F17" t="n">
-        <v>30</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>-1077</v>
+        <v>331</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>2101.85</v>
       </c>
       <c r="H17" t="n">
-        <v>-1.11</v>
+        <v>2.1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>SL HIT</t>
+          <t>TARGET HIT</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1280,33 +1280,33 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>PAGEIND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5450</v>
+        <v>40885</v>
       </c>
       <c r="E18" t="n">
-        <v>5381.9</v>
+        <v>41702.7</v>
       </c>
       <c r="F18" t="n">
-        <v>18</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>-1225.8</v>
+        <v>2</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>1635.4</v>
       </c>
       <c r="H18" t="n">
-        <v>-1.25</v>
+        <v>2</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>SL HIT</t>
+          <t>TARGET HIT</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1341,19 +1341,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>151.72</v>
+        <v>1852.4</v>
       </c>
       <c r="E19" t="n">
-        <v>150.19</v>
+        <v>1833.88</v>
       </c>
       <c r="F19" t="n">
-        <v>659</v>
+        <v>53</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-1008.27</v>
+        <v>-981.5599999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>-1.01</v>
+        <v>-1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1367,14 +1367,14 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>BULLISH</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>CHOLAFIN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1388,19 +1388,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1120</v>
+        <v>1799.6</v>
       </c>
       <c r="E20" t="n">
-        <v>1155.25</v>
+        <v>1781.6</v>
       </c>
       <c r="F20" t="n">
-        <v>89</v>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>3137.25</v>
+        <v>55</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>-990</v>
       </c>
       <c r="H20" t="n">
-        <v>3.15</v>
+        <v>-1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1409,45 +1409,45 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>TARGET HIT</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>BULLISH</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
       <c r="D21" t="n">
-        <v>620.1</v>
+        <v>1385.3</v>
       </c>
       <c r="E21" t="n">
-        <v>610.45</v>
+        <v>1371.45</v>
       </c>
       <c r="F21" t="n">
-        <v>161</v>
+        <v>72</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-1553.65</v>
+        <v>-997.2</v>
       </c>
       <c r="H21" t="n">
-        <v>-1.56</v>
+        <v>-1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1461,14 +1461,14 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>BULLISH</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1482,19 +1482,19 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>302</v>
+        <v>959.85</v>
       </c>
       <c r="E22" t="n">
-        <v>308.35</v>
+        <v>950.25</v>
       </c>
       <c r="F22" t="n">
-        <v>331</v>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>2101.85</v>
+        <v>104</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>-998.4</v>
       </c>
       <c r="H22" t="n">
-        <v>2.1</v>
+        <v>-1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>TARGET HIT</t>
+          <t>SL HIT</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1763,244 +1763,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PAGEIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40885</v>
+        <v>1455.4</v>
       </c>
       <c r="D6" t="n">
-        <v>41370</v>
+        <v>1465.4</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="F6" t="n">
-        <v>81770</v>
+        <v>98967.2</v>
       </c>
       <c r="G6" t="n">
-        <v>970</v>
+        <v>680</v>
       </c>
       <c r="H6" t="n">
-        <v>1.19</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>40476.15</v>
+        <v>1440.85</v>
       </c>
       <c r="J6" t="n">
-        <v>41702.7</v>
+        <v>1484.51</v>
       </c>
       <c r="K6" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GODREJPROP</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1852.4</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1866.6</v>
-      </c>
-      <c r="E7" t="n">
-        <v>53</v>
-      </c>
-      <c r="F7" t="n">
-        <v>98177.2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>752.6</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1833.88</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1889.45</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CHOLAFIN</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1799.6</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1789.8</v>
-      </c>
-      <c r="E8" t="n">
-        <v>55</v>
-      </c>
-      <c r="F8" t="n">
-        <v>98978</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-539</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1781.6</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1835.59</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>UNITDSPR</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>1385.3</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1350.4</v>
-      </c>
-      <c r="E9" t="n">
-        <v>72</v>
-      </c>
-      <c r="F9" t="n">
-        <v>99741.60000000001</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-2512.8</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-2.52</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1371.45</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1413.01</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CIPLA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1455.4</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1465.4</v>
-      </c>
-      <c r="E10" t="n">
-        <v>68</v>
-      </c>
-      <c r="F10" t="n">
-        <v>98967.2</v>
-      </c>
-      <c r="G10" t="n">
-        <v>680</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1440.85</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1484.51</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>959.85</v>
-      </c>
-      <c r="D11" t="n">
-        <v>952.15</v>
-      </c>
-      <c r="E11" t="n">
-        <v>104</v>
-      </c>
-      <c r="F11" t="n">
-        <v>99824.39999999999</v>
-      </c>
-      <c r="G11" t="n">
-        <v>-800.8</v>
-      </c>
-      <c r="H11" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="I11" t="n">
-        <v>950.25</v>
-      </c>
-      <c r="J11" t="n">
-        <v>979.05</v>
-      </c>
-      <c r="K11" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
@@ -2022,7 +1817,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -2073,22 +1868,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2941.5</v>
+        <v>4576.9</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="G2" t="n">
-        <v>2941.5</v>
+        <v>4576.9</v>
       </c>
     </row>
     <row r="3">
@@ -2098,22 +1893,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>903.1799999999999</v>
+        <v>6</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>-2065.58</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>33.3</v>
+        <v>16.7</v>
       </c>
       <c r="G3" t="n">
-        <v>3844.68</v>
+        <v>2511.32</v>
       </c>
     </row>
     <row r="4">
@@ -2123,22 +1918,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>548.2</v>
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>-450.2</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="G4" t="n">
-        <v>4392.88</v>
+        <v>2061.12</v>
       </c>
     </row>
   </sheetData>
@@ -2157,7 +1952,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -2208,22 +2003,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2941.5</v>
+        <v>4576.9</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="G2" t="n">
-        <v>2941.5</v>
+        <v>4576.9</v>
       </c>
     </row>
     <row r="3">
@@ -2233,22 +2028,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1451.38</v>
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>-2515.78</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
-        <v>40</v>
+        <v>22.2</v>
       </c>
       <c r="G3" t="n">
-        <v>4392.88</v>
+        <v>2061.12</v>
       </c>
     </row>
   </sheetData>
@@ -2318,22 +2113,22 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2061.12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
         <v>11</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>4392.88</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" t="n">
-        <v>7</v>
-      </c>
       <c r="F2" t="n">
-        <v>36.4</v>
+        <v>31.2</v>
       </c>
       <c r="G2" t="n">
-        <v>4392.88</v>
+        <v>2061.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(trader): add scanner entry params to portfolio and Excel
Persist price_chg, oi_chg, vol_ratio, pcr, and sector at entry,
carry them through to closed trades, and export as columns in All
Trades and Open Positions sheets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/trade_log.xlsx
+++ b/trade_log.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -461,11 +461,16 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,27 +506,52 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Price Chg %</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>OI Chg %</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Vol Ratio</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>PCR</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Exit Reason</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
         </is>
       </c>
     </row>
@@ -545,30 +575,51 @@
         <v>1577.8</v>
       </c>
       <c r="E2" t="n">
-        <v>1578.7</v>
+        <v>1608.2</v>
       </c>
       <c r="F2" t="n">
         <v>63</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>56.7</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H2" t="n">
-        <v>0.06</v>
+        <v>13.47</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>1915.2</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -592,30 +643,51 @@
         <v>14098</v>
       </c>
       <c r="E3" t="n">
-        <v>14115</v>
+        <v>14442</v>
       </c>
       <c r="F3" t="n">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>119</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H3" t="n">
-        <v>0.12</v>
+        <v>10.44</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>2408</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -639,30 +711,51 @@
         <v>330.1</v>
       </c>
       <c r="E4" t="n">
-        <v>330.05</v>
+        <v>328.75</v>
       </c>
       <c r="F4" t="n">
         <v>302</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>-15.1</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>-0.02</v>
+        <v>8.58</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>-407.7</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -686,30 +779,51 @@
         <v>714.15</v>
       </c>
       <c r="E5" t="n">
-        <v>713.95</v>
+        <v>738.85</v>
       </c>
       <c r="F5" t="n">
         <v>140</v>
       </c>
-      <c r="G5" s="4" t="n">
-        <v>-28</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>-0.03</v>
+        <v>4.76</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>3458</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -733,30 +847,55 @@
         <v>1455.4</v>
       </c>
       <c r="E6" t="n">
-        <v>1465.4</v>
+        <v>1458</v>
       </c>
       <c r="F6" t="n">
         <v>68</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>680</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.6899999999999999</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -785,25 +924,50 @@
       <c r="F7" t="n">
         <v>93</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>-1469.4</v>
       </c>
-      <c r="H7" t="n">
+      <c r="N7" t="n">
         <v>-1.48</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -832,25 +996,50 @@
       <c r="F8" t="n">
         <v>9</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="n">
         <v>3028.5</v>
       </c>
-      <c r="H8" t="n">
+      <c r="N8" t="n">
         <v>3.21</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>TARGET HIT</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -879,25 +1068,50 @@
       <c r="F9" t="n">
         <v>19</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="n">
         <v>4423.2</v>
       </c>
-      <c r="H9" t="n">
+      <c r="N9" t="n">
         <v>4.47</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>TARGET HIT</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -926,25 +1140,50 @@
       <c r="F10" t="n">
         <v>252</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>-1108.8</v>
       </c>
-      <c r="H10" t="n">
+      <c r="N10" t="n">
         <v>-1.11</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -973,25 +1212,50 @@
       <c r="F11" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>-855</v>
       </c>
-      <c r="H11" t="n">
+      <c r="N11" t="n">
         <v>-1.09</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1020,25 +1284,50 @@
       <c r="F12" t="n">
         <v>30</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>-1077</v>
       </c>
-      <c r="H12" t="n">
+      <c r="N12" t="n">
         <v>-1.11</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1067,25 +1356,50 @@
       <c r="F13" t="n">
         <v>18</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>-1225.8</v>
       </c>
-      <c r="H13" t="n">
+      <c r="N13" t="n">
         <v>-1.25</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1114,25 +1428,50 @@
       <c r="F14" t="n">
         <v>659</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>-1008.27</v>
       </c>
-      <c r="H14" t="n">
+      <c r="N14" t="n">
         <v>-1.01</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1161,25 +1500,50 @@
       <c r="F15" t="n">
         <v>89</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="n">
         <v>3137.25</v>
       </c>
-      <c r="H15" t="n">
+      <c r="N15" t="n">
         <v>3.15</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>TARGET HIT</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1208,25 +1572,50 @@
       <c r="F16" t="n">
         <v>161</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="n">
         <v>-1553.65</v>
       </c>
-      <c r="H16" t="n">
+      <c r="N16" t="n">
         <v>-1.56</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1255,25 +1644,50 @@
       <c r="F17" t="n">
         <v>331</v>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="n">
         <v>2101.85</v>
       </c>
-      <c r="H17" t="n">
+      <c r="N17" t="n">
         <v>2.1</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>TARGET HIT</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1302,25 +1716,50 @@
       <c r="F18" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="n">
         <v>1635.4</v>
       </c>
-      <c r="H18" t="n">
+      <c r="N18" t="n">
         <v>2</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>TARGET HIT</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1349,25 +1788,50 @@
       <c r="F19" t="n">
         <v>53</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="n">
         <v>-981.5599999999999</v>
       </c>
-      <c r="H19" t="n">
+      <c r="N19" t="n">
         <v>-1</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
         </is>
       </c>
     </row>
@@ -1396,25 +1860,50 @@
       <c r="F20" t="n">
         <v>55</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>-990</v>
       </c>
-      <c r="H20" t="n">
+      <c r="N20" t="n">
         <v>-1</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
         </is>
       </c>
     </row>
@@ -1443,25 +1932,50 @@
       <c r="F21" t="n">
         <v>72</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="n">
         <v>-997.2</v>
       </c>
-      <c r="H21" t="n">
+      <c r="N21" t="n">
         <v>-1</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
         </is>
       </c>
     </row>
@@ -1490,25 +2004,50 @@
       <c r="F22" t="n">
         <v>104</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>-998.4</v>
       </c>
-      <c r="H22" t="n">
+      <c r="N22" t="n">
         <v>-1</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>SL HIT</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1523,20 +2062,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1557,42 +2101,67 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Price Chg %</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>OI Chg %</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Vol Ratio</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>PCR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
           <t>CMP ₹</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Invested ₹</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Unrealised ₹</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>SL ₹</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Target ₹</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
         </is>
       </c>
     </row>
@@ -1610,31 +2179,52 @@
       <c r="C2" t="n">
         <v>1577.8</v>
       </c>
-      <c r="D2" t="n">
-        <v>1578.7</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E2" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1608.2</v>
+      </c>
+      <c r="K2" t="n">
         <v>63</v>
       </c>
-      <c r="F2" t="n">
+      <c r="L2" t="n">
         <v>99401.39999999999</v>
       </c>
-      <c r="G2" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="M2" t="n">
+        <v>1915.2</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="O2" t="n">
         <v>1562.02</v>
       </c>
-      <c r="J2" t="n">
+      <c r="P2" t="n">
         <v>1609.36</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -1651,31 +2241,52 @@
       <c r="C3" t="n">
         <v>14098</v>
       </c>
-      <c r="D3" t="n">
-        <v>14115</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E3" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>14442</v>
+      </c>
+      <c r="K3" t="n">
         <v>7</v>
       </c>
-      <c r="F3" t="n">
+      <c r="L3" t="n">
         <v>98686</v>
       </c>
-      <c r="G3" t="n">
-        <v>119</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="I3" t="n">
+      <c r="M3" t="n">
+        <v>2408</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="O3" t="n">
         <v>13957.02</v>
       </c>
-      <c r="J3" t="n">
+      <c r="P3" t="n">
         <v>14379.96</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
       </c>
     </row>
     <row r="4">
@@ -1692,31 +2303,52 @@
       <c r="C4" t="n">
         <v>330.1</v>
       </c>
-      <c r="D4" t="n">
-        <v>330.05</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E4" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>328.75</v>
+      </c>
+      <c r="K4" t="n">
         <v>302</v>
       </c>
-      <c r="F4" t="n">
+      <c r="L4" t="n">
         <v>99690.2</v>
       </c>
-      <c r="G4" t="n">
-        <v>-15.1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="M4" t="n">
+        <v>-407.7</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="O4" t="n">
         <v>326.8</v>
       </c>
-      <c r="J4" t="n">
+      <c r="P4" t="n">
         <v>336.7</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
       </c>
     </row>
     <row r="5">
@@ -1733,31 +2365,52 @@
       <c r="C5" t="n">
         <v>714.15</v>
       </c>
-      <c r="D5" t="n">
-        <v>713.95</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E5" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>738.85</v>
+      </c>
+      <c r="K5" t="n">
         <v>140</v>
       </c>
-      <c r="F5" t="n">
+      <c r="L5" t="n">
         <v>99981</v>
       </c>
-      <c r="G5" t="n">
-        <v>-28</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="M5" t="n">
+        <v>3458</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="O5" t="n">
         <v>707.01</v>
       </c>
-      <c r="J5" t="n">
+      <c r="P5" t="n">
         <v>728.4299999999999</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
       </c>
     </row>
     <row r="6">
@@ -1774,31 +2427,56 @@
       <c r="C6" t="n">
         <v>1455.4</v>
       </c>
-      <c r="D6" t="n">
-        <v>1465.4</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1458</v>
+      </c>
+      <c r="K6" t="n">
         <v>68</v>
       </c>
-      <c r="F6" t="n">
+      <c r="L6" t="n">
         <v>98967.2</v>
       </c>
-      <c r="G6" t="n">
-        <v>680</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="M6" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="O6" t="n">
         <v>1440.85</v>
       </c>
-      <c r="J6" t="n">
+      <c r="P6" t="n">
         <v>1484.51</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>